<commit_message>
Deploy Atlas site from 02ce5070a8f5ba25a59fc6e2aa95dcda0bf23322
</commit_message>
<xml_diff>
--- a/downloads/artifacts/stakeholder-power-interest-grid/stakeholder-power-interest-grid-example.xlsx
+++ b/downloads/artifacts/stakeholder-power-interest-grid/stakeholder-power-interest-grid-example.xlsx
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="J5" s="4">
-        <f>IF(OR(H5="",I5=""),"",IF(AND(H5="High",I5="High"),"Manage closely",IF(AND(H5="High",I5="Low"),"Keep satisfied",IF(AND(H5="Low",I5="High"),"Keep informed","Monitor"))))</f>
+        <f>IF(OR(H5="",I5=""),"",IF(AND(H5="High",I5="High"),"Manage Closely",IF(AND(H5="High",I5="Low"),"Keep Satisfied",IF(AND(H5="Low",I5="High"),"Keep Informed","Monitor"))))</f>
         <v/>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="J6" s="5">
-        <f>IF(OR(H6="",I6=""),"",IF(AND(H6="High",I6="High"),"Manage closely",IF(AND(H6="High",I6="Low"),"Keep satisfied",IF(AND(H6="Low",I6="High"),"Keep informed","Monitor"))))</f>
+        <f>IF(OR(H6="",I6=""),"",IF(AND(H6="High",I6="High"),"Manage Closely",IF(AND(H6="High",I6="Low"),"Keep Satisfied",IF(AND(H6="Low",I6="High"),"Keep Informed","Monitor"))))</f>
         <v/>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="J7" s="4">
-        <f>IF(OR(H7="",I7=""),"",IF(AND(H7="High",I7="High"),"Manage closely",IF(AND(H7="High",I7="Low"),"Keep satisfied",IF(AND(H7="Low",I7="High"),"Keep informed","Monitor"))))</f>
+        <f>IF(OR(H7="",I7=""),"",IF(AND(H7="High",I7="High"),"Manage Closely",IF(AND(H7="High",I7="Low"),"Keep Satisfied",IF(AND(H7="Low",I7="High"),"Keep Informed","Monitor"))))</f>
         <v/>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="J8" s="5">
-        <f>IF(OR(H8="",I8=""),"",IF(AND(H8="High",I8="High"),"Manage closely",IF(AND(H8="High",I8="Low"),"Keep satisfied",IF(AND(H8="Low",I8="High"),"Keep informed","Monitor"))))</f>
+        <f>IF(OR(H8="",I8=""),"",IF(AND(H8="High",I8="High"),"Manage Closely",IF(AND(H8="High",I8="Low"),"Keep Satisfied",IF(AND(H8="Low",I8="High"),"Keep Informed","Monitor"))))</f>
         <v/>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="J9" s="4">
-        <f>IF(OR(H9="",I9=""),"",IF(AND(H9="High",I9="High"),"Manage closely",IF(AND(H9="High",I9="Low"),"Keep satisfied",IF(AND(H9="Low",I9="High"),"Keep informed","Monitor"))))</f>
+        <f>IF(OR(H9="",I9=""),"",IF(AND(H9="High",I9="High"),"Manage Closely",IF(AND(H9="High",I9="Low"),"Keep Satisfied",IF(AND(H9="Low",I9="High"),"Keep Informed","Monitor"))))</f>
         <v/>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1118,7 +1118,7 @@
         </is>
       </c>
       <c r="J10" s="5">
-        <f>IF(OR(H10="",I10=""),"",IF(AND(H10="High",I10="High"),"Manage closely",IF(AND(H10="High",I10="Low"),"Keep satisfied",IF(AND(H10="Low",I10="High"),"Keep informed","Monitor"))))</f>
+        <f>IF(OR(H10="",I10=""),"",IF(AND(H10="High",I10="High"),"Manage Closely",IF(AND(H10="High",I10="Low"),"Keep Satisfied",IF(AND(H10="Low",I10="High"),"Keep Informed","Monitor"))))</f>
         <v/>
       </c>
       <c r="K10" s="5" t="inlineStr">

</xml_diff>